<commit_message>
fix: räknesnurra 1–1000 säljare och fler snabbval
Föreningar kan räkna 1–1 000 säljare och välja 300/500 medlemmar
samt 2 000/3 000 kr i snitt. Enkelhets-slides in i kommunikations-
och föreningsdeck.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/presentations/Roots_Raknesnurra.xlsx
+++ b/docs/presentations/Roots_Raknesnurra.xlsx
@@ -78,43 +78,43 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <color rgb="001D1D1B"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00D5CABF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="48"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00EDF1E9"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001D1D1B"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="006B794F"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="007F715B"/>
       <sz val="9"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <color rgb="001D1D1B"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00D5CABF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="48"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <color rgb="00EDF1E9"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="001D1D1B"/>
-      <sz val="18"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="006B794F"/>
-      <sz val="18"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -250,7 +250,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -273,36 +273,35 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="6" fillId="6" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="11" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="14" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="13" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -808,7 +807,7 @@
       <c r="D7" s="4" t="n"/>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>SNABBVAL — klicka och kopiera</t>
+          <t>SNABBVAL — skriv in till vänster</t>
         </is>
       </c>
       <c r="F7" s="7" t="n"/>
@@ -827,32 +826,30 @@
       <c r="D8" s="4" t="n"/>
       <c r="E8" s="11" t="inlineStr">
         <is>
-          <t>Storlek</t>
-        </is>
-      </c>
-      <c r="F8" s="12" t="inlineStr">
-        <is>
-          <t>Skriv in →</t>
-        </is>
+          <t>Litet lag</t>
+        </is>
+      </c>
+      <c r="F8" s="12" t="n">
+        <v>20</v>
       </c>
       <c r="G8" s="4" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n"/>
-      <c r="B9" s="12" t="inlineStr">
-        <is>
-          <t>Antal medlemmar som säljer (5, 10, 15 …)</t>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>Antal medlemmar som säljer (1–1 000)</t>
         </is>
       </c>
       <c r="C9" s="7" t="n"/>
       <c r="D9" s="4" t="n"/>
-      <c r="E9" s="13" t="inlineStr">
-        <is>
-          <t>Litet lag</t>
-        </is>
-      </c>
-      <c r="F9" s="14" t="n">
-        <v>20</v>
+      <c r="E9" s="11" t="inlineStr">
+        <is>
+          <t>Vanligt</t>
+        </is>
+      </c>
+      <c r="F9" s="12" t="n">
+        <v>50</v>
       </c>
       <c r="G9" s="4" t="n"/>
     </row>
@@ -863,54 +860,54 @@
           <t>Hur mycket säljer var och en?</t>
         </is>
       </c>
-      <c r="C10" s="15" t="n">
+      <c r="C10" s="14" t="n">
         <v>1500</v>
       </c>
       <c r="D10" s="4" t="n"/>
-      <c r="E10" s="13" t="inlineStr">
-        <is>
-          <t>Vanligt</t>
-        </is>
-      </c>
-      <c r="F10" s="14" t="n">
-        <v>50</v>
+      <c r="E10" s="11" t="inlineStr">
+        <is>
+          <t>Stort</t>
+        </is>
+      </c>
+      <c r="F10" s="12" t="n">
+        <v>100</v>
       </c>
       <c r="G10" s="4" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n"/>
-      <c r="B11" s="12" t="inlineStr">
+      <c r="B11" s="13" t="inlineStr">
         <is>
           <t>Snitt per person under kampanjen (max 5 000 kr)</t>
         </is>
       </c>
       <c r="C11" s="7" t="n"/>
       <c r="D11" s="4" t="n"/>
-      <c r="E11" s="13" t="inlineStr">
-        <is>
-          <t>Stort</t>
-        </is>
-      </c>
-      <c r="F11" s="14" t="n">
-        <v>100</v>
+      <c r="E11" s="11" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="F11" s="12" t="n">
+        <v>200</v>
       </c>
       <c r="G11" s="4" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n"/>
-      <c r="B12" s="16">
+      <c r="B12" s="15">
         <f>CONCATENATE("≈ ",ROUND(C10/399,0)," Premiumpaket à 399 kr")</f>
         <v/>
       </c>
       <c r="C12" s="7" t="n"/>
       <c r="D12" s="4" t="n"/>
-      <c r="E12" s="13" t="inlineStr">
-        <is>
-          <t>Mycket stort</t>
-        </is>
-      </c>
-      <c r="F12" s="14" t="n">
-        <v>200</v>
+      <c r="E12" s="11" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="F12" s="12" t="n">
+        <v>300</v>
       </c>
       <c r="G12" s="4" t="n"/>
     </row>
@@ -919,13 +916,19 @@
       <c r="B13" s="4" t="n"/>
       <c r="C13" s="4" t="n"/>
       <c r="D13" s="4" t="n"/>
-      <c r="E13" s="4" t="n"/>
-      <c r="F13" s="4" t="n"/>
+      <c r="E13" s="11" t="inlineStr">
+        <is>
+          <t>500</t>
+        </is>
+      </c>
+      <c r="F13" s="12" t="n">
+        <v>500</v>
+      </c>
       <c r="G13" s="4" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n"/>
-      <c r="B14" s="17" t="inlineStr">
+      <c r="B14" s="16" t="inlineStr">
         <is>
           <t>ER FÖRENING FÅR</t>
         </is>
@@ -934,7 +937,7 @@
     </row>
     <row r="15" ht="28" customHeight="1">
       <c r="A15" s="4" t="n"/>
-      <c r="B15" s="18">
+      <c r="B15" s="17">
         <f>ROUND(C8*C10*0.35,0)</f>
         <v/>
       </c>
@@ -950,7 +953,7 @@
     </row>
     <row r="18" ht="24" customHeight="1">
       <c r="A18" s="4" t="n"/>
-      <c r="B18" s="19">
+      <c r="B18" s="18">
         <f>CONCATENATE("35 % av ",TEXT(C8*C10,"#,##0")," kr i total försäljning")</f>
         <v/>
       </c>
@@ -967,19 +970,19 @@
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="4" t="n"/>
-      <c r="B20" s="20" t="inlineStr">
+      <c r="B20" s="19" t="inlineStr">
         <is>
           <t>Total försäljning</t>
         </is>
       </c>
-      <c r="C20" s="21" t="n"/>
-      <c r="D20" s="20" t="inlineStr">
+      <c r="C20" s="20" t="n"/>
+      <c r="D20" s="19" t="inlineStr">
         <is>
           <t>Per säljare till er</t>
         </is>
       </c>
-      <c r="E20" s="21" t="n"/>
-      <c r="F20" s="20" t="inlineStr">
+      <c r="E20" s="20" t="n"/>
+      <c r="F20" s="19" t="inlineStr">
         <is>
           <t>Er andel</t>
         </is>
@@ -988,15 +991,15 @@
     </row>
     <row r="21" ht="32" customHeight="1">
       <c r="A21" s="4" t="n"/>
-      <c r="B21" s="22">
+      <c r="B21" s="21">
         <f>C8*C10</f>
         <v/>
       </c>
-      <c r="D21" s="22">
+      <c r="D21" s="21">
         <f>IF(C8=0,0,ROUND(C8*C10*0.35/C8,0))</f>
         <v/>
       </c>
-      <c r="F21" s="23" t="inlineStr">
+      <c r="F21" s="22" t="inlineStr">
         <is>
           <t>35 %</t>
         </is>
@@ -1005,16 +1008,16 @@
     </row>
     <row r="22" ht="8" customHeight="1">
       <c r="A22" s="4" t="n"/>
-      <c r="B22" s="21" t="n"/>
-      <c r="C22" s="21" t="n"/>
-      <c r="D22" s="21" t="n"/>
-      <c r="E22" s="21" t="n"/>
-      <c r="F22" s="21" t="n"/>
+      <c r="B22" s="20" t="n"/>
+      <c r="C22" s="20" t="n"/>
+      <c r="D22" s="20" t="n"/>
+      <c r="E22" s="20" t="n"/>
+      <c r="F22" s="20" t="n"/>
       <c r="G22" s="4" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n"/>
-      <c r="B23" s="24" t="inlineStr">
+      <c r="B23" s="23" t="inlineStr">
         <is>
           <t>EXEMPEL NI KAN JÄMFÖRA MED</t>
         </is>
@@ -1023,103 +1026,103 @@
     </row>
     <row r="24">
       <c r="A24" s="4" t="n"/>
-      <c r="B24" s="25" t="inlineStr"/>
-      <c r="C24" s="25" t="inlineStr">
+      <c r="B24" s="24" t="inlineStr"/>
+      <c r="C24" s="24" t="inlineStr">
         <is>
           <t>Medlemmar</t>
         </is>
       </c>
-      <c r="D24" s="25" t="inlineStr">
+      <c r="D24" s="24" t="inlineStr">
         <is>
           <t>Snitt/person</t>
         </is>
       </c>
-      <c r="E24" s="25" t="inlineStr">
+      <c r="E24" s="24" t="inlineStr">
         <is>
           <t>Ni får</t>
         </is>
       </c>
-      <c r="F24" s="25" t="inlineStr"/>
+      <c r="F24" s="24" t="inlineStr"/>
       <c r="G24" s="4" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n"/>
-      <c r="B25" s="26" t="inlineStr">
+      <c r="B25" s="25" t="inlineStr">
         <is>
           <t>Litet lag</t>
         </is>
       </c>
-      <c r="C25" s="27" t="n">
+      <c r="C25" s="26" t="n">
         <v>20</v>
       </c>
-      <c r="D25" s="28" t="n">
+      <c r="D25" s="27" t="n">
         <v>1000</v>
       </c>
-      <c r="E25" s="29">
+      <c r="E25" s="28">
         <f>ROUND(C25*D25*0.35,0)</f>
         <v/>
       </c>
-      <c r="F25" s="21" t="n"/>
+      <c r="F25" s="20" t="n"/>
       <c r="G25" s="4" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="4" t="n"/>
-      <c r="B26" s="26" t="inlineStr">
+      <c r="B26" s="25" t="inlineStr">
         <is>
           <t>Vanlig förening</t>
         </is>
       </c>
-      <c r="C26" s="27" t="n">
+      <c r="C26" s="26" t="n">
         <v>50</v>
       </c>
-      <c r="D26" s="28" t="n">
+      <c r="D26" s="27" t="n">
         <v>1500</v>
       </c>
-      <c r="E26" s="29">
+      <c r="E26" s="28">
         <f>ROUND(C26*D26*0.35,0)</f>
         <v/>
       </c>
-      <c r="F26" s="21" t="n"/>
+      <c r="F26" s="20" t="n"/>
       <c r="G26" s="4" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n"/>
-      <c r="B27" s="26" t="inlineStr">
+      <c r="B27" s="25" t="inlineStr">
         <is>
           <t>Stark kampanj</t>
         </is>
       </c>
-      <c r="C27" s="27" t="n">
+      <c r="C27" s="26" t="n">
         <v>100</v>
       </c>
-      <c r="D27" s="28" t="n">
+      <c r="D27" s="27" t="n">
         <v>2500</v>
       </c>
-      <c r="E27" s="29">
+      <c r="E27" s="28">
         <f>ROUND(C27*D27*0.35,0)</f>
         <v/>
       </c>
-      <c r="F27" s="21" t="n"/>
+      <c r="F27" s="20" t="n"/>
       <c r="G27" s="4" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="4" t="n"/>
-      <c r="B28" s="26" t="inlineStr">
+      <c r="B28" s="25" t="inlineStr">
         <is>
           <t>Högt snitt</t>
         </is>
       </c>
-      <c r="C28" s="27" t="n">
+      <c r="C28" s="26" t="n">
         <v>50</v>
       </c>
-      <c r="D28" s="28" t="n">
+      <c r="D28" s="27" t="n">
         <v>5000</v>
       </c>
-      <c r="E28" s="29">
+      <c r="E28" s="28">
         <f>ROUND(C28*D28*0.35,0)</f>
         <v/>
       </c>
-      <c r="F28" s="21" t="n"/>
+      <c r="F28" s="20" t="n"/>
       <c r="G28" s="4" t="n"/>
     </row>
     <row r="29">
@@ -1133,7 +1136,7 @@
     </row>
     <row r="30" ht="32" customHeight="1">
       <c r="A30" s="4" t="n"/>
-      <c r="B30" s="30" t="inlineStr">
+      <c r="B30" s="29" t="inlineStr">
         <is>
           <t>Tips: Premiumpaketet kostar 399 kr — då går ca 140 kr till föreningen per paket. Öppna fliken »Så funkar det« om ni vill förstå mer.  ·  info@roots.nu  ·  roots.nu</t>
         </is>
@@ -1150,13 +1153,13 @@
       <c r="G31" s="4" t="n"/>
     </row>
     <row r="32" ht="22" customHeight="1">
-      <c r="A32" s="31" t="n"/>
-      <c r="B32" s="32" t="inlineStr">
+      <c r="A32" s="30" t="n"/>
+      <c r="B32" s="31" t="inlineStr">
         <is>
           <t>Roots  ·  Räknesnurra för föreningar  ·  35 % låst andel</t>
         </is>
       </c>
-      <c r="G32" s="31" t="n"/>
+      <c r="G32" s="30" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="n"/>
@@ -1197,13 +1200,13 @@
   </mergeCells>
   <conditionalFormatting sqref="C8">
     <cfRule type="expression" priority="1" dxfId="0">
-      <formula>MOD(C8,5)&lt;&gt;0</formula>
+      <formula>OR(C8&lt;1,C8&gt;1000)</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="C8" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="Ogiltigt" error="Ange mellan 5 och 2 000 (helst 5-tal)." promptTitle="Medlemmar" prompt="Välj ett jämnt 5-tal, t.ex. 20, 50 eller 100." type="whole" operator="between">
-      <formula1>5</formula1>
-      <formula2>2000</formula2>
+    <dataValidation sqref="C8" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="Ogiltigt" error="Ange ett heltal mellan 1 och 1 000." promptTitle="Medlemmar" prompt="Ange hur många som säljer (1–1 000)." type="whole" operator="between">
+      <formula1>1</formula1>
+      <formula2>1000</formula2>
     </dataValidation>
     <dataValidation sqref="C10" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="För högt" error="Max 5 000 kr per säljare." promptTitle="Snittförsäljning" prompt="Max 5 000 kr per person under kampanjen." type="whole" operator="between">
       <formula1>0</formula1>
@@ -1237,7 +1240,7 @@
     </row>
     <row r="2" ht="36" customHeight="1">
       <c r="A2" s="1" t="n"/>
-      <c r="B2" s="33" t="inlineStr">
+      <c r="B2" s="32" t="inlineStr">
         <is>
           <t>Så funkar räknesnurran</t>
         </is>
@@ -1256,7 +1259,7 @@
     </row>
     <row r="5">
       <c r="A5" s="4" t="n"/>
-      <c r="B5" s="34" t="inlineStr">
+      <c r="B5" s="33" t="inlineStr">
         <is>
           <t>Tre steg</t>
         </is>
@@ -1265,9 +1268,9 @@
     </row>
     <row r="6" ht="55" customHeight="1">
       <c r="A6" s="4" t="n"/>
-      <c r="B6" s="35" t="inlineStr">
-        <is>
-          <t>1) Skriv hur många som säljer (jämna 5-tal).
+      <c r="B6" s="34" t="inlineStr">
+        <is>
+          <t>1) Skriv hur många som säljer (1–1 000).
 2) Skriv hur mycket varje person säljer för i snitt.
 3) Läs av den stora gröna siffran — det är vad föreningen får.</t>
         </is>
@@ -1291,7 +1294,7 @@
     </row>
     <row r="10">
       <c r="A10" s="4" t="n"/>
-      <c r="B10" s="34" t="inlineStr">
+      <c r="B10" s="33" t="inlineStr">
         <is>
           <t>Formeln</t>
         </is>
@@ -1300,7 +1303,7 @@
     </row>
     <row r="11" ht="55" customHeight="1">
       <c r="A11" s="4" t="n"/>
-      <c r="B11" s="35" t="inlineStr">
+      <c r="B11" s="34" t="inlineStr">
         <is>
           <t>Medlemmar × snittförsäljning × 35 % = föreningens förtjänst.
 Exempel: 50 × 1 500 kr × 35 % = 26 250 kr till er.</t>
@@ -1320,7 +1323,7 @@
     </row>
     <row r="14">
       <c r="A14" s="4" t="n"/>
-      <c r="B14" s="34" t="inlineStr">
+      <c r="B14" s="33" t="inlineStr">
         <is>
           <t>Varför 35 %?</t>
         </is>
@@ -1329,7 +1332,7 @@
     </row>
     <row r="15" ht="55" customHeight="1">
       <c r="A15" s="4" t="n"/>
-      <c r="B15" s="35" t="inlineStr">
+      <c r="B15" s="34" t="inlineStr">
         <is>
           <t>Andelen är låst i Roots-erbjudandet — samma siffra i portalen, avräkningen och den här filen. Ingen förhandling, inga dolda avdrag.</t>
         </is>
@@ -1348,7 +1351,7 @@
     </row>
     <row r="18">
       <c r="A18" s="4" t="n"/>
-      <c r="B18" s="34" t="inlineStr">
+      <c r="B18" s="33" t="inlineStr">
         <is>
           <t>Premiumpaketet</t>
         </is>
@@ -1357,7 +1360,7 @@
     </row>
     <row r="19" ht="55" customHeight="1">
       <c r="A19" s="4" t="n"/>
-      <c r="B19" s="35" t="inlineStr">
+      <c r="B19" s="34" t="inlineStr">
         <is>
           <t>Paketpris 399 kr (schampo + balsam + body wash).
 Ca 140 kr går till föreningen per sålt paket.</t>
@@ -1377,7 +1380,7 @@
     </row>
     <row r="22">
       <c r="A22" s="4" t="n"/>
-      <c r="B22" s="34" t="inlineStr">
+      <c r="B22" s="33" t="inlineStr">
         <is>
           <t>Behöver ni hjälp?</t>
         </is>
@@ -1386,7 +1389,7 @@
     </row>
     <row r="23" ht="55" customHeight="1">
       <c r="A23" s="4" t="n"/>
-      <c r="B23" s="35" t="inlineStr">
+      <c r="B23" s="34" t="inlineStr">
         <is>
           <t>Mejla info@roots.nu eller gå till roots.nu — vi räknar gärna live med er.</t>
         </is>

</xml_diff>